<commit_message>
Update the email outline spreadsheet
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/email/email-outline.xlsx
+++ b/docs/email/email-outline.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\lmslocal\docs\email\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEB09729-29A4-41B7-B0D4-EBEE1F613DE7}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D07D741-CF80-445E-B2FD-A45166776CF3}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8940" xr2:uid="{04AC65AE-6C17-448A-A5A6-78B888B68FDF}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="29">
   <si>
     <t>Join Comp</t>
   </si>
@@ -93,9 +93,6 @@
     <t>Result set mid round</t>
   </si>
   <si>
-    <t>MOBILE NOTIFICATION</t>
-  </si>
-  <si>
     <t>Y</t>
   </si>
   <si>
@@ -106,6 +103,15 @@
   </si>
   <si>
     <t>Game started</t>
+  </si>
+  <si>
+    <t>BUILT</t>
+  </si>
+  <si>
+    <t>MOBILE NOTIFICATION (pending)</t>
+  </si>
+  <si>
+    <t>--</t>
   </si>
 </sst>
 </file>
@@ -170,12 +176,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -492,18 +501,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E8D174EA-1CB0-4AAB-99E9-FB17E825ADF7}">
-  <dimension ref="B2:E17"/>
+  <dimension ref="B2:F17"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="16" style="1" customWidth="1"/>
     <col min="3" max="3" width="17.5546875" style="1" customWidth="1"/>
     <col min="4" max="4" width="24.88671875" style="1" customWidth="1"/>
-    <col min="5" max="5" width="21.77734375" style="1" customWidth="1"/>
+    <col min="6" max="6" width="32.33203125" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B2" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>15</v>
@@ -512,10 +521,13 @@
         <v>16</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="3" spans="2:5" x14ac:dyDescent="0.3">
+        <v>26</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="3" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B3" s="1" t="s">
         <v>4</v>
       </c>
@@ -525,11 +537,11 @@
       <c r="D3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="E3" s="1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="4" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="F3" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="4" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B4" s="1" t="s">
         <v>4</v>
       </c>
@@ -540,10 +552,13 @@
         <v>2</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="5" spans="2:5" x14ac:dyDescent="0.3">
+        <v>22</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="5" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B5" s="1" t="s">
         <v>4</v>
       </c>
@@ -553,8 +568,11 @@
       <c r="D5" s="1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="6" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="F5" s="3" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="6" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B6" s="1" t="s">
         <v>5</v>
       </c>
@@ -564,8 +582,11 @@
       <c r="D6" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="7" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="F6" s="3" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="7" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B7" s="1" t="s">
         <v>5</v>
       </c>
@@ -575,8 +596,11 @@
       <c r="D7" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="8" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="F7" s="3" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="8" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B8" s="1" t="s">
         <v>5</v>
       </c>
@@ -586,8 +610,11 @@
       <c r="D8" s="1" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="9" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="F8" s="3" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="9" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B9" s="1" t="s">
         <v>10</v>
       </c>
@@ -597,8 +624,11 @@
       <c r="D9" s="1" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="10" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="F9" s="3" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="10" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B10" s="1" t="s">
         <v>5</v>
       </c>
@@ -608,8 +638,11 @@
       <c r="D10" s="1" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="11" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="F10" s="3" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="11" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B11" s="1" t="s">
         <v>5</v>
       </c>
@@ -619,8 +652,11 @@
       <c r="D11" s="1" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="12" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="F11" s="3" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="12" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B12" s="1" t="s">
         <v>10</v>
       </c>
@@ -630,8 +666,11 @@
       <c r="D12" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="13" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="F12" s="3" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="13" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B13" s="1" t="s">
         <v>4</v>
       </c>
@@ -641,8 +680,11 @@
       <c r="D13" s="1" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="14" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="F13" s="3" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="14" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B14" s="1" t="s">
         <v>5</v>
       </c>
@@ -652,8 +694,11 @@
       <c r="D14" s="1" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="15" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="F14" s="3" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="15" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B15" s="1" t="s">
         <v>10</v>
       </c>
@@ -663,8 +708,11 @@
       <c r="D15" s="1" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="16" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="F15" s="3" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="16" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B16" s="1" t="s">
         <v>4</v>
       </c>
@@ -672,13 +720,13 @@
         <v>18</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="E16" s="1" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="17" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="F16" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="17" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B17" s="1" t="s">
         <v>4</v>
       </c>
@@ -686,10 +734,10 @@
         <v>18</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="E17" s="1" t="s">
-        <v>23</v>
+        <v>25</v>
+      </c>
+      <c r="F17" s="1" t="s">
+        <v>22</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Broadcast off the Emails table, and no status column
Broadcast from Organiser was dropped rather than deferred, so its
mapping in emailPreference.js goes with it - a mapping kept "in case"
outlives the memory of why, and if it is ever revived the mapping
belongs in the same commit as the sender.

Broadcast from Admin has its own screen, so its row on the Emails table
was a permanently "Not wired" line whose only content was a pointer to
the button already in the header.

With both gone every remaining row is built, and the Status column said
"Ready" eleven times. Dropping it takes `wired` with it: no greyed rows,
no dimmed names, and Preview subject only to the competition rule. The
server still refuses an unbuilt type with UNSUPPORTED_EMAIL_TYPE, so
this table was never the thing stopping a bad send.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/email/email-outline.xlsx
+++ b/docs/email/email-outline.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\lmslocal\docs\email\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF8CF077-792F-4EA3-8366-D2848ADBB8DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E636F24-1B52-4543-B860-F28240DFB26C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{04AC65AE-6C17-448A-A5A6-78B888B68FDF}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="25">
   <si>
     <t>Round Over</t>
   </si>
@@ -94,12 +94,6 @@
   </si>
   <si>
     <t>Broadcast from Admin</t>
-  </si>
-  <si>
-    <t>Broadcast from Organiser</t>
-  </si>
-  <si>
-    <t>Game Members</t>
   </si>
   <si>
     <t>BROADCAST</t>
@@ -173,7 +167,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -182,6 +176,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -498,7 +495,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E8D174EA-1CB0-4AAB-99E9-FB17E825ADF7}">
-  <dimension ref="B2:F16"/>
+  <dimension ref="B2:F15"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="22.21875" style="1" customWidth="1"/>
@@ -634,7 +631,7 @@
         <v>12</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="E9" s="1" t="s">
         <v>13</v>
@@ -651,7 +648,7 @@
         <v>12</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="E10" s="1" t="s">
         <v>13</v>
@@ -713,7 +710,7 @@
     </row>
     <row r="14" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B14" s="2" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C14" s="2"/>
       <c r="D14" s="2"/>
@@ -730,21 +727,10 @@
       <c r="D15" s="1" t="s">
         <v>21</v>
       </c>
+      <c r="E15" s="4" t="s">
+        <v>13</v>
+      </c>
       <c r="F15" s="3" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="16" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B16" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="C16" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="D16" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="F16" s="3" t="s">
         <v>17</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Put share_reminder on the outline, and a deploy note
email-outline.xlsx is the authoritative list of what we send, and share_reminder
was built without a row on it - the one loose end flagged when it landed. The
README section describing its rules can stop being a proposal now that the
outline agrees.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/email/email-outline.xlsx
+++ b/docs/email/email-outline.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\lmslocal\docs\email\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E636F24-1B52-4543-B860-F28240DFB26C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C548DC71-4D62-4BFC-A8E0-CDB7F8EEA789}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{04AC65AE-6C17-448A-A5A6-78B888B68FDF}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="26">
   <si>
     <t>Round Over</t>
   </si>
@@ -103,6 +103,9 @@
   </si>
   <si>
     <t>Hint - Result set mid round</t>
+  </si>
+  <si>
+    <t>Share reminder</t>
   </si>
 </sst>
 </file>
@@ -495,7 +498,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E8D174EA-1CB0-4AAB-99E9-FB17E825ADF7}">
-  <dimension ref="B2:F15"/>
+  <dimension ref="B2:F16"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="22.21875" style="1" customWidth="1"/>
@@ -659,13 +662,13 @@
     </row>
     <row r="11" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B11" s="1" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="E11" s="1" t="s">
         <v>13</v>
@@ -676,13 +679,13 @@
     </row>
     <row r="12" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B12" s="1" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>12</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E12" s="1" t="s">
         <v>13</v>
@@ -693,44 +696,61 @@
     </row>
     <row r="13" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B13" s="1" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F13" s="3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="14" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B14" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D14" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="E13" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="F13" s="3" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="14" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B14" s="2" t="s">
+      <c r="E14" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="15" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B15" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="C14" s="2"/>
-      <c r="D14" s="2"/>
-      <c r="E14" s="2"/>
-      <c r="F14" s="2"/>
-    </row>
-    <row r="15" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B15" s="1" t="s">
+      <c r="C15" s="2"/>
+      <c r="D15" s="2"/>
+      <c r="E15" s="2"/>
+      <c r="F15" s="2"/>
+    </row>
+    <row r="16" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B16" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C15" s="1" t="s">
+      <c r="C16" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="D15" s="1" t="s">
+      <c r="D16" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="E15" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="F15" s="3" t="s">
+      <c r="E16" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F16" s="3" t="s">
         <v>17</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Drop Game Start reminder
Unwired, the second email dropped today and for the same reason as
share_reminder. It chased an organiser whose fixture-service competition could
start but who had never pressed Ready.

The state has not vanished: 207 was created on 8 Aug with no start block, so it
has no rounds and no ready_at, and it would have qualified on 22 Aug once past
the 14-day threshold. It is dropped because email is the wrong instrument - an
organiser who has not pressed a button in a fortnight is disengaged, and email
is what disengaged people ignore. A dashboard notice reaches them where they
are looking.

Service and template stay on disk. The note records what is worth keeping if it
is ever revived: candidates ran through getCompetitionStartOutlook, the same
function behind the organiser's own start card, so nobody was chased toward a
button that would then refuse them.

Catalog down to 10 wired emails, all carded.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/email/email-outline.xlsx
+++ b/docs/email/email-outline.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\lmslocal\docs\email\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0469A970-3C54-48EB-9BB5-80C3A89BE2CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B11E8447-709B-49A3-9E8D-622664D29C3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{04AC65AE-6C17-448A-A5A6-78B888B68FDF}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="24">
   <si>
     <t>Round Over</t>
   </si>
@@ -49,9 +49,6 @@
   </si>
   <si>
     <t>Fixture reminder</t>
-  </si>
-  <si>
-    <t>Game Start reminder</t>
   </si>
   <si>
     <t>All</t>
@@ -495,7 +492,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E8D174EA-1CB0-4AAB-99E9-FB17E825ADF7}">
-  <dimension ref="B2:F15"/>
+  <dimension ref="B2:F14"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="22.21875" style="1" customWidth="1"/>
@@ -506,19 +503,19 @@
   <sheetData>
     <row r="2" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E2" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="C2" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="E2" s="2" t="s">
+      <c r="F2" s="2" t="s">
         <v>15</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="3" spans="2:6" x14ac:dyDescent="0.3">
@@ -526,16 +523,16 @@
         <v>3</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>0</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4" spans="2:6" x14ac:dyDescent="0.3">
@@ -543,16 +540,16 @@
         <v>3</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>1</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="5" spans="2:6" x14ac:dyDescent="0.3">
@@ -560,16 +557,16 @@
         <v>3</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>2</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="6" spans="2:6" x14ac:dyDescent="0.3">
@@ -577,16 +574,16 @@
         <v>4</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="7" spans="2:6" x14ac:dyDescent="0.3">
@@ -594,16 +591,16 @@
         <v>4</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="8" spans="2:6" x14ac:dyDescent="0.3">
@@ -614,13 +611,13 @@
         <v>11</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>6</v>
+        <v>22</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="9" spans="2:6" x14ac:dyDescent="0.3">
@@ -628,108 +625,91 @@
         <v>4</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D9" s="1" t="s">
         <v>23</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="10" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B10" s="1" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="11" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B11" s="1" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D11" s="1" t="s">
         <v>18</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="12" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B12" s="1" t="s">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D12" s="1" t="s">
         <v>19</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="13" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B13" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="D13" s="1" t="s">
+      <c r="B13" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C13" s="2"/>
+      <c r="D13" s="2"/>
+      <c r="E13" s="2"/>
+      <c r="F13" s="2"/>
+    </row>
+    <row r="14" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B14" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D14" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="E13" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="F13" s="3" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="14" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B14" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="C14" s="2"/>
-      <c r="D14" s="2"/>
-      <c r="E14" s="2"/>
-      <c r="F14" s="2"/>
-    </row>
-    <row r="15" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B15" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C15" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="D15" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="E15" s="4"/>
-      <c r="F15" s="3" t="s">
-        <v>17</v>
+      <c r="E14" s="4"/>
+      <c r="F14" s="3" t="s">
+        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add the outline row for the cron work
Andreas's own edit to the authoritative outline, kept separate from the code
commit it belongs to so the spreadsheet's history stays readable on its own.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/email/email-outline.xlsx
+++ b/docs/email/email-outline.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\lmslocal\docs\email\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFBD7F33-645B-4E05-B2BE-745FAD5DE8B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CDE45D1-BCA0-4F98-9127-730CD6DB8318}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{04AC65AE-6C17-448A-A5A6-78B888B68FDF}"/>
   </bookViews>
@@ -102,7 +102,7 @@
     <t>Hint - Result set mid round</t>
   </si>
   <si>
-    <t>Nudge after join and quiet</t>
+    <t>Empty competition</t>
   </si>
 </sst>
 </file>
@@ -676,7 +676,7 @@
     </row>
     <row r="12" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B12" s="1" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>11</v>

</xml_diff>